<commit_message>
Final work hours excel
</commit_message>
<xml_diff>
--- a/docs/Työajan seuranta Arttu.xlsx
+++ b/docs/Työajan seuranta Arttu.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arttu\Dropbox\Koulu\Web-ohjelmoinnin sovellusprojekti\Movieproject\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD7651FC-8442-4F72-884C-9D6D4AD89732}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC9C255F-E9A6-4B81-9AAA-42F6CDBC5E3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3345" yWindow="5955" windowWidth="17670" windowHeight="11790" xr2:uid="{B7036960-D674-4B76-B564-D076AACD5E6B}"/>
+    <workbookView xWindow="3345" yWindow="5955" windowWidth="17670" windowHeight="9870" xr2:uid="{B7036960-D674-4B76-B564-D076AACD5E6B}"/>
   </bookViews>
   <sheets>
     <sheet name="Arttu Jämsä" sheetId="3" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
   <si>
     <t>Ryhmä:</t>
   </si>
@@ -156,6 +156,15 @@
   </si>
   <si>
     <t>Palaverit koko ajalta</t>
+  </si>
+  <si>
+    <t>10.10.</t>
+  </si>
+  <si>
+    <t>PR korjausta</t>
+  </si>
+  <si>
+    <t>Yht:</t>
   </si>
 </sst>
 </file>
@@ -511,7 +520,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C1EECD9-4AD3-41AF-8923-B28678799497}">
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.85546875" customWidth="1"/>
@@ -519,7 +528,7 @@
     <col min="3" max="3" width="11.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -527,7 +536,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -537,8 +546,11 @@
       <c r="C2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="E2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>38</v>
       </c>
@@ -546,10 +558,14 @@
         <v>39</v>
       </c>
       <c r="C3">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+      <c r="E3">
+        <f>SUM(C3:C27)</f>
+        <v>63</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -560,7 +576,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -571,7 +587,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
@@ -582,7 +598,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
@@ -593,7 +609,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -604,7 +620,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>14</v>
       </c>
@@ -615,7 +631,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -626,7 +642,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>18</v>
       </c>
@@ -637,7 +653,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>20</v>
       </c>
@@ -648,7 +664,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>22</v>
       </c>
@@ -659,7 +675,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>23</v>
       </c>
@@ -670,7 +686,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>26</v>
       </c>
@@ -734,6 +750,17 @@
       </c>
       <c r="C21">
         <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>40</v>
+      </c>
+      <c r="B22" t="s">
+        <v>41</v>
+      </c>
+      <c r="C22">
+        <v>0.5</v>
       </c>
     </row>
   </sheetData>
@@ -742,6 +769,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="44038759-07ae-40d4-bc3d-7c9fb0b3775b" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009BAF6AFB37B6774A9122C6036818BC92" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c611cd0fe7e35dfe638a44e659100205">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="44038759-07ae-40d4-bc3d-7c9fb0b3775b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="36a43d4c38ea7f7b42b5de64d2c1c906" ns3:_="">
     <xsd:import namespace="44038759-07ae-40d4-bc3d-7c9fb0b3775b"/>
@@ -921,14 +956,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="44038759-07ae-40d4-bc3d-7c9fb0b3775b" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -939,6 +966,16 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D3DBD177-6275-4D31-B82C-61F9284D9B7B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="44038759-07ae-40d4-bc3d-7c9fb0b3775b"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B52374CD-1656-483C-BC7A-A879F7105755}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -956,16 +993,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D3DBD177-6275-4D31-B82C-61F9284D9B7B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="44038759-07ae-40d4-bc3d-7c9fb0b3775b"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{28C42445-4535-4827-89B5-92D7D04A90E8}">
   <ds:schemaRefs>

</xml_diff>